<commit_message>
Update reports 2026-09-30 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-30.xlsx
+++ b/gex_pivot_levels_2026-09-30.xlsx
@@ -573,12 +573,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$22.95M</t>
+          <t>-$16.26M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$41.82M</t>
+          <t>+$29.62M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -593,215 +593,219 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>7697.91</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>7625</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="A4" s="5" t="n">
+        <v>7711.63</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>761</v>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>-$179.15M</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>+$232.61M</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>7717.91</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>7645</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-$15.29M</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>+$19.12M</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>7711.63</v>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>761</v>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>-$179.15M</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>+$232.61M</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>+$1.43M</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>+$12.35M</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>7717.91</v>
+        <v>7721.67</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>7645</v>
+        <v>762</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-$1.26M</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>+$22.76M</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>7722.91</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>7650</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>+$1.83M</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>+$15.76M</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>7721.67</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>762</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>-$22.01M</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>+$47.26M</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7747.91</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7675</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>-$5.53M</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>+$55.42M</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>7751.78</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>765</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>-$1.26M</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>+$22.76M</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>7722.91</v>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>-$27.09M</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>+$58.17M</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>-$39.88M</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>+$96.41M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>7747.91</v>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>7675</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>-$5.81M</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>+$58.26M</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>7751.78</v>
+        <v>7762.91</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>765</v>
+        <v>7690</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>-$39.88M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>+$66.50M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$96.41M</t>
+          <t>+$79.46M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -811,16 +815,16 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>7762.91</v>
+        <v>7772.91</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>7690</v>
+        <v>7700</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -829,12 +833,12 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>+$62.81M</t>
+          <t>+$1.18M</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>+$75.04M</t>
+          <t>+$152.96M</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -844,16 +848,16 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>7772.91</v>
+        <v>7792.91</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>7700</v>
+        <v>7720</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -862,20 +866,24 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>+$1.04M</t>
+          <t>+$15.82M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$134.87M</t>
+          <t>+$22.88M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -891,12 +899,12 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>+$2.71M</t>
+          <t>+$3.66M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$26.10M</t>
+          <t>+$35.26M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -949,12 +957,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>+$8.64M</t>
+          <t>+$12.65M</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$31.17M</t>
+          <t>+$45.65M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -2976,38 +2984,42 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="5" t="n">
         <v>7772.91</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="5" t="n">
         <v>7700</v>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>+$1.04M</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>+$134.87M</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>+$1.18M</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>+$152.96M</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3180,12 +3192,12 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>+$62.81M</t>
+          <t>+$66.50M</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>+$75.04M</t>
+          <t>+$79.46M</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -3274,28 +3286,28 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>7747.91</v>
+        <v>2867.1</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>7675</v>
+        <v>285</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>-$5.81M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>+$7.01M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>+$58.26M</t>
+          <t>+$56.98M</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3308,28 +3320,28 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>7722.91</v>
+        <v>30898.93</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>7650</v>
+        <v>745</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>-$27.09M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>+$47.03M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>+$58.17M</t>
+          <t>+$55.65M</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -3339,35 +3351,35 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>2867.1</v>
+        <v>7747.91</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>285</v>
+        <v>7675</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>+$7.01M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>-$5.53M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>+$56.98M</t>
+          <t>+$55.42M</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -3384,10 +3396,10 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>30898.93</v>
+        <v>30693.36</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -3396,12 +3408,12 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>+$47.03M</t>
+          <t>+$23.99M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>+$55.65M</t>
+          <t>+$49.73M</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -3418,28 +3430,28 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>30693.36</v>
+        <v>7722.91</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>740</v>
+        <v>7650</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>+$23.99M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>-$22.01M</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>+$49.73M</t>
+          <t>+$47.26M</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -3449,7 +3461,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3492,42 +3504,38 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
-        <v>7672.91</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>7600</v>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="B18" s="2" t="n">
+        <v>7822.91</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>-$22.95M</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>+$41.82M</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>+$12.65M</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>+$45.65M</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -3570,10 +3578,10 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7822.91</v>
+        <v>7797.91</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>7750</v>
+        <v>7725</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
@@ -3582,12 +3590,12 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>+$8.64M</t>
+          <t>+$3.66M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$31.17M</t>
+          <t>+$35.26M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -3600,100 +3608,104 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>7672.91</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>7600</v>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>-$16.26M</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>+$29.62M</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B22" s="5" t="n">
         <v>29871.07</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C22" s="5" t="n">
         <v>720</v>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>-$19.03M</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>+$28.38M</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>7852.16</v>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>775</v>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>+$13.69M</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>+$28.01M</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>2786.62</v>
+        <v>7852.16</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>277</v>
+        <v>775</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>-$27.01M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>+$13.69M</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+$27.72M</t>
+          <t>+$28.01M</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -3706,28 +3718,28 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>7797.91</v>
+        <v>2786.62</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>7725</v>
+        <v>277</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>+$2.71M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>-$27.01M</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>+$26.10M</t>
+          <t>+$27.72M</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -3782,24 +3794,24 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>7721.67</v>
+        <v>7792.91</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>762</v>
+        <v>7720</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>-$1.26M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>+$15.82M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>+$22.76M</t>
+          <t>+$22.88M</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -3820,32 +3832,36 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>7697.91</v>
+        <v>7721.67</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>7625</v>
+        <v>762</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>-$15.29M</t>
+          <t>-$1.26M</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>+$19.12M</t>
+          <t>+$22.76M</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -3958,78 +3974,78 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>87.55</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>-$12.79M</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>+$12.89M</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B32" s="2" t="n">
         <v>7717.91</v>
       </c>
-      <c r="C31" s="2" t="n">
+      <c r="C32" s="2" t="n">
         <v>7645</v>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>+$1.83M</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>+$15.76M</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>+$1.43M</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>+$12.35M</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>87.55</v>
-      </c>
-      <c r="C32" s="5" t="n">
-        <v>140</v>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>-$12.79M</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>+$12.89M</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>

</xml_diff>